<commit_message>
Regenerate all four cuisines under ADR 0007
`python scripts/run.py --all` on the committed caches. No fetch, no scrape, no
row added or removed: 201 / 154 / 24 / 31 rows in and out.

Fields that move anywhere in the scored JSON are composite_rating,
adjusted_rating, value_score, the two percentiles, sources, n_sources, and
google_wilson (nulled when its rating is excluded), plus the new
google_trusted and excluded_sources. Everything else is byte-identical —
closed, closed_override, business_status, coordinates, neighborhood_raw,
raw_rating, review_count and place_id all unchanged, and the closed counts
hold at 26 / 8 / 0 / 0.

Kensington has no untrusted match at all, so it gains the two annotation
fields and nothing else.

The four root .xlsx files also gain an "Excluded Sources" column, on top of
their usual openpyxl timestamp churn.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TY45ZGTCTuV5EWpmZziADv
</commit_message>
<xml_diff>
--- a/Italian_Ratings.xlsx
+++ b/Italian_Ratings.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Italian" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Italian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P155"/>
+  <dimension ref="A1:Q155"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,7 @@
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
     <col width="35" customWidth="1" min="16" max="16"/>
+    <col width="60" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -526,6 +527,11 @@
       <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Google Maps Name</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Excluded Sources</t>
         </is>
       </c>
     </row>
@@ -566,13 +572,13 @@
         <v>4.325</v>
       </c>
       <c r="L2" t="n">
-        <v>91.5</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="M2" t="n">
         <v>4.482</v>
       </c>
       <c r="N2" t="n">
-        <v>83</v>
+        <v>84.2</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
@@ -580,6 +586,7 @@
           <t>Via Carota</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -618,13 +625,13 @@
         <v>4.302</v>
       </c>
       <c r="L3" t="n">
-        <v>86.90000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="M3" t="n">
         <v>4.261</v>
       </c>
       <c r="N3" t="n">
-        <v>58.2</v>
+        <v>59.9</v>
       </c>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
@@ -632,6 +639,7 @@
           <t>Don Angie</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -670,13 +678,13 @@
         <v>4.205</v>
       </c>
       <c r="L4" t="n">
-        <v>78.40000000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="M4" t="n">
         <v>4.165</v>
       </c>
       <c r="N4" t="n">
-        <v>45.1</v>
+        <v>46.7</v>
       </c>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
@@ -684,6 +692,7 @@
           <t>San Sabino</t>
         </is>
       </c>
+      <c r="Q4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -722,13 +731,13 @@
         <v>4.318</v>
       </c>
       <c r="L5" t="n">
-        <v>90.2</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="M5" t="n">
         <v>4.364</v>
       </c>
       <c r="N5" t="n">
-        <v>66.7</v>
+        <v>67.8</v>
       </c>
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
@@ -736,6 +745,7 @@
           <t>L'Artusi</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -774,13 +784,13 @@
         <v>4.232</v>
       </c>
       <c r="L6" t="n">
-        <v>80.40000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="M6" t="n">
         <v>4.254</v>
       </c>
       <c r="N6" t="n">
-        <v>55.6</v>
+        <v>56.6</v>
       </c>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
@@ -788,6 +798,7 @@
           <t>I Sodi</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -826,13 +837,13 @@
         <v>4.004</v>
       </c>
       <c r="L7" t="n">
-        <v>35.3</v>
+        <v>38.2</v>
       </c>
       <c r="M7" t="n">
         <v>4.447</v>
       </c>
       <c r="N7" t="n">
-        <v>77.09999999999999</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
@@ -840,6 +851,7 @@
           <t>Bar Pisellino</t>
         </is>
       </c>
+      <c r="Q7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -884,7 +896,7 @@
         <v>3.961</v>
       </c>
       <c r="N8" t="n">
-        <v>15.7</v>
+        <v>15.8</v>
       </c>
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
@@ -892,6 +904,7 @@
           <t>Gene's</t>
         </is>
       </c>
+      <c r="Q8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -930,13 +943,13 @@
         <v>3.964</v>
       </c>
       <c r="L9" t="n">
-        <v>26.1</v>
+        <v>28.9</v>
       </c>
       <c r="M9" t="n">
         <v>4.08</v>
       </c>
       <c r="N9" t="n">
-        <v>32.7</v>
+        <v>34.2</v>
       </c>
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
@@ -944,6 +957,7 @@
           <t>Villa Mosconi Restaurant</t>
         </is>
       </c>
+      <c r="Q9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -982,13 +996,13 @@
         <v>4.177</v>
       </c>
       <c r="L10" t="n">
-        <v>77.09999999999999</v>
+        <v>78.3</v>
       </c>
       <c r="M10" t="n">
         <v>4.068</v>
       </c>
       <c r="N10" t="n">
-        <v>28.8</v>
+        <v>30.3</v>
       </c>
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
@@ -996,6 +1010,7 @@
           <t>Babbo</t>
         </is>
       </c>
+      <c r="Q10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1034,13 +1049,13 @@
         <v>3.896</v>
       </c>
       <c r="L11" t="n">
-        <v>14.4</v>
+        <v>17.1</v>
       </c>
       <c r="M11" t="n">
         <v>4.009</v>
       </c>
       <c r="N11" t="n">
-        <v>21.6</v>
+        <v>23</v>
       </c>
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
@@ -1048,6 +1063,7 @@
           <t>Lupa</t>
         </is>
       </c>
+      <c r="Q11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1086,13 +1102,13 @@
         <v>4.276</v>
       </c>
       <c r="L12" t="n">
-        <v>84.3</v>
+        <v>85.5</v>
       </c>
       <c r="M12" t="n">
         <v>4.08</v>
       </c>
       <c r="N12" t="n">
-        <v>32</v>
+        <v>33.6</v>
       </c>
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
@@ -1100,6 +1116,7 @@
           <t>Carbone New York</t>
         </is>
       </c>
+      <c r="Q12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1138,13 +1155,13 @@
         <v>4.138</v>
       </c>
       <c r="L13" t="n">
-        <v>71.90000000000001</v>
+        <v>73.7</v>
       </c>
       <c r="M13" t="n">
         <v>4.259</v>
       </c>
       <c r="N13" t="n">
-        <v>57.5</v>
+        <v>59.2</v>
       </c>
       <c r="O13" t="inlineStr"/>
       <c r="P13" t="inlineStr">
@@ -1152,6 +1169,7 @@
           <t>Emilio's Ballato</t>
         </is>
       </c>
+      <c r="Q13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1190,13 +1208,13 @@
         <v>4.312</v>
       </c>
       <c r="L14" t="n">
-        <v>89.5</v>
+        <v>90.8</v>
       </c>
       <c r="M14" t="n">
         <v>4.67</v>
       </c>
       <c r="N14" t="n">
-        <v>90.2</v>
+        <v>90.8</v>
       </c>
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
@@ -1204,6 +1222,7 @@
           <t>Rubirosa</t>
         </is>
       </c>
+      <c r="Q14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1242,13 +1261,13 @@
         <v>4.065</v>
       </c>
       <c r="L15" t="n">
-        <v>54.2</v>
+        <v>56.6</v>
       </c>
       <c r="M15" t="n">
         <v>3.904</v>
       </c>
       <c r="N15" t="n">
-        <v>11.8</v>
+        <v>12.5</v>
       </c>
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
@@ -1256,6 +1275,7 @@
           <t>Torrisi</t>
         </is>
       </c>
+      <c r="Q15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1294,13 +1314,13 @@
         <v>3.975</v>
       </c>
       <c r="L16" t="n">
-        <v>29.4</v>
+        <v>32.2</v>
       </c>
       <c r="M16" t="n">
         <v>3.903</v>
       </c>
       <c r="N16" t="n">
-        <v>11.1</v>
+        <v>11.8</v>
       </c>
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
@@ -1308,6 +1328,7 @@
           <t>Roscioli NYC</t>
         </is>
       </c>
+      <c r="Q16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1346,13 +1367,13 @@
         <v>3.856</v>
       </c>
       <c r="L17" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="M17" t="n">
         <v>3.968</v>
       </c>
       <c r="N17" t="n">
-        <v>17</v>
+        <v>17.1</v>
       </c>
       <c r="O17" t="inlineStr"/>
       <c r="P17" t="inlineStr">
@@ -1360,6 +1381,7 @@
           <t>Bar Pitti</t>
         </is>
       </c>
+      <c r="Q17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1398,13 +1420,13 @@
         <v>3.957</v>
       </c>
       <c r="L18" t="n">
-        <v>25.5</v>
+        <v>28.3</v>
       </c>
       <c r="M18" t="n">
         <v>4.072</v>
       </c>
       <c r="N18" t="n">
-        <v>30.7</v>
+        <v>32.2</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
@@ -1412,6 +1434,7 @@
           <t>Sant Ambroeus West Village</t>
         </is>
       </c>
+      <c r="Q18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1450,13 +1473,13 @@
         <v>4.052</v>
       </c>
       <c r="L19" t="n">
-        <v>51</v>
+        <v>53.9</v>
       </c>
       <c r="M19" t="n">
         <v>4.171</v>
       </c>
       <c r="N19" t="n">
-        <v>46.4</v>
+        <v>48</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="inlineStr">
@@ -1464,6 +1487,7 @@
           <t>Malaparte</t>
         </is>
       </c>
+      <c r="Q19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1502,13 +1526,13 @@
         <v>4.115</v>
       </c>
       <c r="L20" t="n">
-        <v>66</v>
+        <v>67.8</v>
       </c>
       <c r="M20" t="n">
         <v>4.009</v>
       </c>
       <c r="N20" t="n">
-        <v>20.9</v>
+        <v>22.4</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
@@ -1516,6 +1540,7 @@
           <t>da Toscano</t>
         </is>
       </c>
+      <c r="Q20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1554,13 +1579,13 @@
         <v>4.176</v>
       </c>
       <c r="L21" t="n">
-        <v>76.5</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="M21" t="n">
         <v>4.577</v>
       </c>
       <c r="N21" t="n">
-        <v>89.5</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="inlineStr">
@@ -1568,6 +1593,7 @@
           <t>Fiaschetteria “Pistoia”</t>
         </is>
       </c>
+      <c r="Q21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1612,7 +1638,7 @@
         <v>4.576</v>
       </c>
       <c r="N22" t="n">
-        <v>88.90000000000001</v>
+        <v>89.5</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
@@ -1620,6 +1646,7 @@
           <t>Osteria Nonnino</t>
         </is>
       </c>
+      <c r="Q22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1658,13 +1685,13 @@
         <v>3.767</v>
       </c>
       <c r="L23" t="n">
-        <v>6.5</v>
+        <v>6.6</v>
       </c>
       <c r="M23" t="n">
         <v>3.877</v>
       </c>
       <c r="N23" t="n">
-        <v>8.5</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
@@ -1672,6 +1699,7 @@
           <t>Arthur and Sons NY Italian</t>
         </is>
       </c>
+      <c r="Q23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1710,13 +1738,13 @@
         <v>3.834</v>
       </c>
       <c r="L24" t="n">
-        <v>8.5</v>
+        <v>8.6</v>
       </c>
       <c r="M24" t="n">
         <v>3.946</v>
       </c>
       <c r="N24" t="n">
-        <v>15</v>
+        <v>15.1</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
@@ -1724,6 +1752,7 @@
           <t>Frankies 570 Spuntino</t>
         </is>
       </c>
+      <c r="Q24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1776,6 +1805,7 @@
           <t>Da Andrea Greenwich Village</t>
         </is>
       </c>
+      <c r="Q25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1811,21 +1841,26 @@
         <v>631</v>
       </c>
       <c r="K26" t="n">
-        <v>4.023</v>
+        <v>3.852</v>
       </c>
       <c r="L26" t="n">
-        <v>41.8</v>
+        <v>9.9</v>
       </c>
       <c r="M26" t="n">
-        <v>3.919</v>
+        <v>3.753</v>
       </c>
       <c r="N26" t="n">
-        <v>13.1</v>
+        <v>3.3</v>
       </c>
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
           <t>Il Mulino - Downtown (West 3rd)</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>Google rating 4.5 excluded — Google returned 'Il Mulino - Downtown (West 3rd)', whose name similarity to 'Il Mulino New York' is 0.58 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -1880,6 +1915,7 @@
           <t>OLIO E PIÙ</t>
         </is>
       </c>
+      <c r="Q27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1918,13 +1954,13 @@
         <v>4.304</v>
       </c>
       <c r="L28" t="n">
-        <v>88.2</v>
+        <v>89.5</v>
       </c>
       <c r="M28" t="n">
         <v>4.717</v>
       </c>
       <c r="N28" t="n">
-        <v>92.8</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
@@ -1932,6 +1968,7 @@
           <t>Lavagna</t>
         </is>
       </c>
+      <c r="Q28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1970,13 +2007,13 @@
         <v>4.266</v>
       </c>
       <c r="L29" t="n">
-        <v>82.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="M29" t="n">
         <v>4.39</v>
       </c>
       <c r="N29" t="n">
-        <v>70.59999999999999</v>
+        <v>71.7</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr">
@@ -1984,6 +2021,7 @@
           <t>Il Posto Accanto</t>
         </is>
       </c>
+      <c r="Q29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2022,13 +2060,13 @@
         <v>4.01</v>
       </c>
       <c r="L30" t="n">
-        <v>37.3</v>
+        <v>40.1</v>
       </c>
       <c r="M30" t="n">
         <v>4.127</v>
       </c>
       <c r="N30" t="n">
-        <v>39.9</v>
+        <v>41.4</v>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="inlineStr">
@@ -2036,6 +2074,7 @@
           <t>Supper</t>
         </is>
       </c>
+      <c r="Q30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2088,6 +2127,7 @@
           <t>Cacio e Pepe</t>
         </is>
       </c>
+      <c r="Q31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2126,13 +2166,13 @@
         <v>3.981</v>
       </c>
       <c r="L32" t="n">
-        <v>30.7</v>
+        <v>33.6</v>
       </c>
       <c r="M32" t="n">
         <v>4.098</v>
       </c>
       <c r="N32" t="n">
-        <v>35.3</v>
+        <v>36.8</v>
       </c>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr">
@@ -2140,6 +2180,7 @@
           <t>John's of 12th Street</t>
         </is>
       </c>
+      <c r="Q32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2178,13 +2219,13 @@
         <v>4.215</v>
       </c>
       <c r="L33" t="n">
-        <v>79.09999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="M33" t="n">
         <v>4.338</v>
       </c>
       <c r="N33" t="n">
-        <v>65.40000000000001</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="O33" t="inlineStr"/>
       <c r="P33" t="inlineStr">
@@ -2192,6 +2233,7 @@
           <t>Forsythia NYC</t>
         </is>
       </c>
+      <c r="Q33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2236,7 +2278,7 @@
         <v>3.774</v>
       </c>
       <c r="N34" t="n">
-        <v>3.3</v>
+        <v>3.9</v>
       </c>
       <c r="O34" t="inlineStr"/>
       <c r="P34" t="inlineStr">
@@ -2244,6 +2286,7 @@
           <t>Una Pizza Napoletana</t>
         </is>
       </c>
+      <c r="Q34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2282,13 +2325,13 @@
         <v>4.019</v>
       </c>
       <c r="L35" t="n">
-        <v>39.9</v>
+        <v>42.8</v>
       </c>
       <c r="M35" t="n">
         <v>4.77</v>
       </c>
       <c r="N35" t="n">
-        <v>95.40000000000001</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr">
@@ -2296,6 +2339,7 @@
           <t>Scarr's Pizza</t>
         </is>
       </c>
+      <c r="Q35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2334,13 +2378,13 @@
         <v>3.953</v>
       </c>
       <c r="L36" t="n">
-        <v>24.2</v>
+        <v>27</v>
       </c>
       <c r="M36" t="n">
         <v>4.069</v>
       </c>
       <c r="N36" t="n">
-        <v>29.4</v>
+        <v>30.9</v>
       </c>
       <c r="O36" t="inlineStr"/>
       <c r="P36" t="inlineStr">
@@ -2348,6 +2392,7 @@
           <t>Altro Paradiso</t>
         </is>
       </c>
+      <c r="Q36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2392,7 +2437,7 @@
         <v>3.885</v>
       </c>
       <c r="N37" t="n">
-        <v>9.800000000000001</v>
+        <v>10.5</v>
       </c>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr">
@@ -2400,6 +2445,7 @@
           <t>Pasquale Jones</t>
         </is>
       </c>
+      <c r="Q37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2438,13 +2484,13 @@
         <v>3.931</v>
       </c>
       <c r="L38" t="n">
-        <v>20.3</v>
+        <v>23.7</v>
       </c>
       <c r="M38" t="n">
         <v>4.046</v>
       </c>
       <c r="N38" t="n">
-        <v>26.8</v>
+        <v>28.9</v>
       </c>
       <c r="O38" t="inlineStr"/>
       <c r="P38" t="inlineStr">
@@ -2452,6 +2498,7 @@
           <t>Lodi</t>
         </is>
       </c>
+      <c r="Q38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2490,13 +2537,13 @@
         <v>4.004</v>
       </c>
       <c r="L39" t="n">
-        <v>34.6</v>
+        <v>37.5</v>
       </c>
       <c r="M39" t="n">
         <v>4.121</v>
       </c>
       <c r="N39" t="n">
-        <v>37.9</v>
+        <v>39.5</v>
       </c>
       <c r="O39" t="inlineStr"/>
       <c r="P39" t="inlineStr">
@@ -2504,6 +2551,7 @@
           <t>Sandro's</t>
         </is>
       </c>
+      <c r="Q39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2542,13 +2590,13 @@
         <v>4.046</v>
       </c>
       <c r="L40" t="n">
-        <v>47.1</v>
+        <v>50</v>
       </c>
       <c r="M40" t="n">
         <v>4.164</v>
       </c>
       <c r="N40" t="n">
-        <v>43.8</v>
+        <v>45.4</v>
       </c>
       <c r="O40" t="inlineStr"/>
       <c r="P40" t="inlineStr">
@@ -2556,6 +2604,7 @@
           <t>Gelso &amp; Grand</t>
         </is>
       </c>
+      <c r="Q40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2594,13 +2643,13 @@
         <v>4.026</v>
       </c>
       <c r="L41" t="n">
-        <v>42.5</v>
+        <v>45.4</v>
       </c>
       <c r="M41" t="n">
         <v>4.412</v>
       </c>
       <c r="N41" t="n">
-        <v>72.5</v>
+        <v>74.3</v>
       </c>
       <c r="O41" t="inlineStr"/>
       <c r="P41" t="inlineStr">
@@ -2608,6 +2657,7 @@
           <t>Parm Mulberry Street</t>
         </is>
       </c>
+      <c r="Q41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2646,13 +2696,13 @@
         <v>4.129</v>
       </c>
       <c r="L42" t="n">
-        <v>68</v>
+        <v>69.7</v>
       </c>
       <c r="M42" t="n">
         <v>4.249</v>
       </c>
       <c r="N42" t="n">
-        <v>54.9</v>
+        <v>55.9</v>
       </c>
       <c r="O42" t="inlineStr"/>
       <c r="P42" t="inlineStr">
@@ -2660,6 +2710,7 @@
           <t>Café Mars</t>
         </is>
       </c>
+      <c r="Q42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2695,21 +2746,26 @@
         <v>240</v>
       </c>
       <c r="K43" t="n">
-        <v>4.391</v>
+        <v>4.022</v>
       </c>
       <c r="L43" t="n">
-        <v>96.7</v>
+        <v>44.7</v>
       </c>
       <c r="M43" t="n">
-        <v>4.812</v>
+        <v>4.408</v>
       </c>
       <c r="N43" t="n">
-        <v>96.7</v>
+        <v>73.7</v>
       </c>
       <c r="O43" t="inlineStr"/>
       <c r="P43" t="inlineStr">
         <is>
           <t>OLIO E PIÙ East Village</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>Google rating 4.9 excluded — Google returned 'OLIO E PIÙ East Village', whose name similarity to 'Olmo' is 0.26 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -2750,13 +2806,13 @@
         <v>3.986</v>
       </c>
       <c r="L44" t="n">
-        <v>32.7</v>
+        <v>35.5</v>
       </c>
       <c r="M44" t="n">
         <v>3.882</v>
       </c>
       <c r="N44" t="n">
-        <v>9.199999999999999</v>
+        <v>9.9</v>
       </c>
       <c r="O44" t="inlineStr"/>
       <c r="P44" t="inlineStr">
@@ -2764,6 +2820,7 @@
           <t>Locanda Verde Tribeca</t>
         </is>
       </c>
+      <c r="Q44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2802,13 +2859,13 @@
         <v>3.898</v>
       </c>
       <c r="L45" t="n">
-        <v>15</v>
+        <v>18.4</v>
       </c>
       <c r="M45" t="n">
         <v>3.797</v>
       </c>
       <c r="N45" t="n">
-        <v>5.2</v>
+        <v>5.9</v>
       </c>
       <c r="O45" t="inlineStr"/>
       <c r="P45" t="inlineStr">
@@ -2816,6 +2873,7 @@
           <t>Borgo</t>
         </is>
       </c>
+      <c r="Q45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2854,13 +2912,13 @@
         <v>4.115</v>
       </c>
       <c r="L46" t="n">
-        <v>65.40000000000001</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="M46" t="n">
         <v>4.235</v>
       </c>
       <c r="N46" t="n">
-        <v>52.9</v>
+        <v>53.9</v>
       </c>
       <c r="O46" t="inlineStr"/>
       <c r="P46" t="inlineStr">
@@ -2868,6 +2926,7 @@
           <t>Briscola Trattoria</t>
         </is>
       </c>
+      <c r="Q46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2910,6 +2969,7 @@
       </c>
       <c r="O47" t="inlineStr"/>
       <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2948,13 +3008,13 @@
         <v>4.27</v>
       </c>
       <c r="L48" t="n">
-        <v>83.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="M48" t="n">
         <v>4.129</v>
       </c>
       <c r="N48" t="n">
-        <v>40.5</v>
+        <v>42.1</v>
       </c>
       <c r="O48" t="inlineStr"/>
       <c r="P48" t="inlineStr">
@@ -2962,6 +3022,7 @@
           <t>Rezdôra</t>
         </is>
       </c>
+      <c r="Q48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3000,13 +3061,13 @@
         <v>4.175</v>
       </c>
       <c r="L49" t="n">
-        <v>75.8</v>
+        <v>77</v>
       </c>
       <c r="M49" t="n">
         <v>4.297</v>
       </c>
       <c r="N49" t="n">
-        <v>62.7</v>
+        <v>63.8</v>
       </c>
       <c r="O49" t="inlineStr"/>
       <c r="P49" t="inlineStr">
@@ -3014,6 +3075,7 @@
           <t>La Pecora Bianca NoMad</t>
         </is>
       </c>
+      <c r="Q49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3052,13 +3114,13 @@
         <v>3.916</v>
       </c>
       <c r="L50" t="n">
-        <v>17</v>
+        <v>20.4</v>
       </c>
       <c r="M50" t="n">
         <v>4.031</v>
       </c>
       <c r="N50" t="n">
-        <v>23.5</v>
+        <v>25.7</v>
       </c>
       <c r="O50" t="inlineStr"/>
       <c r="P50" t="inlineStr">
@@ -3066,6 +3128,7 @@
           <t>Bar Primi Penn District</t>
         </is>
       </c>
+      <c r="Q50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3104,13 +3167,13 @@
         <v>3.896</v>
       </c>
       <c r="L51" t="n">
-        <v>13.7</v>
+        <v>16.4</v>
       </c>
       <c r="M51" t="n">
         <v>3.795</v>
       </c>
       <c r="N51" t="n">
-        <v>4.6</v>
+        <v>5.3</v>
       </c>
       <c r="O51" t="inlineStr"/>
       <c r="P51" t="inlineStr">
@@ -3118,6 +3181,7 @@
           <t>Il Mulino Prime</t>
         </is>
       </c>
+      <c r="Q51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3156,13 +3220,13 @@
         <v>4.015</v>
       </c>
       <c r="L52" t="n">
-        <v>38.6</v>
+        <v>41.4</v>
       </c>
       <c r="M52" t="n">
         <v>3.911</v>
       </c>
       <c r="N52" t="n">
-        <v>12.4</v>
+        <v>13.2</v>
       </c>
       <c r="O52" t="inlineStr"/>
       <c r="P52" t="inlineStr">
@@ -3170,6 +3234,7 @@
           <t>Ai Fiori</t>
         </is>
       </c>
+      <c r="Q52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3208,13 +3273,13 @@
         <v>4.145</v>
       </c>
       <c r="L53" t="n">
-        <v>73.2</v>
+        <v>75</v>
       </c>
       <c r="M53" t="n">
         <v>3.98</v>
       </c>
       <c r="N53" t="n">
-        <v>18.3</v>
+        <v>19.1</v>
       </c>
       <c r="O53" t="inlineStr"/>
       <c r="P53" t="inlineStr">
@@ -3222,6 +3287,7 @@
           <t>Marea</t>
         </is>
       </c>
+      <c r="Q53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3260,13 +3326,13 @@
         <v>4.04</v>
       </c>
       <c r="L54" t="n">
-        <v>45.8</v>
+        <v>48.7</v>
       </c>
       <c r="M54" t="n">
         <v>3.935</v>
       </c>
       <c r="N54" t="n">
-        <v>13.7</v>
+        <v>13.8</v>
       </c>
       <c r="O54" t="inlineStr"/>
       <c r="P54" t="inlineStr">
@@ -3274,6 +3340,7 @@
           <t>Quality Italian</t>
         </is>
       </c>
+      <c r="Q54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3312,13 +3379,13 @@
         <v>4.134</v>
       </c>
       <c r="L55" t="n">
-        <v>69.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="M55" t="n">
         <v>4.027</v>
       </c>
       <c r="N55" t="n">
-        <v>22.2</v>
+        <v>24.3</v>
       </c>
       <c r="O55" t="inlineStr"/>
       <c r="P55" t="inlineStr">
@@ -3326,6 +3393,7 @@
           <t>Patsy's</t>
         </is>
       </c>
+      <c r="Q55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3364,13 +3432,13 @@
         <v>4.091</v>
       </c>
       <c r="L56" t="n">
-        <v>62.1</v>
+        <v>64.5</v>
       </c>
       <c r="M56" t="n">
         <v>3.985</v>
       </c>
       <c r="N56" t="n">
-        <v>19</v>
+        <v>19.7</v>
       </c>
       <c r="O56" t="inlineStr"/>
       <c r="P56" t="inlineStr">
@@ -3378,6 +3446,7 @@
           <t>Massara</t>
         </is>
       </c>
+      <c r="Q56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3416,13 +3485,13 @@
         <v>3.931</v>
       </c>
       <c r="L57" t="n">
-        <v>19</v>
+        <v>22.4</v>
       </c>
       <c r="M57" t="n">
         <v>3.829</v>
       </c>
       <c r="N57" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="O57" t="inlineStr"/>
       <c r="P57" t="inlineStr">
@@ -3430,6 +3499,7 @@
           <t>Bad Roman</t>
         </is>
       </c>
+      <c r="Q57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3468,13 +3538,13 @@
         <v>3.873</v>
       </c>
       <c r="L58" t="n">
-        <v>11.8</v>
+        <v>13.2</v>
       </c>
       <c r="M58" t="n">
         <v>3.986</v>
       </c>
       <c r="N58" t="n">
-        <v>19.6</v>
+        <v>20.4</v>
       </c>
       <c r="O58" t="inlineStr"/>
       <c r="P58" t="inlineStr">
@@ -3482,6 +3552,7 @@
           <t>Giulietta</t>
         </is>
       </c>
+      <c r="Q58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3520,13 +3591,13 @@
         <v>4.39</v>
       </c>
       <c r="L59" t="n">
-        <v>96.09999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="M59" t="n">
         <v>4.276</v>
       </c>
       <c r="N59" t="n">
-        <v>59.5</v>
+        <v>61.2</v>
       </c>
       <c r="O59" t="inlineStr"/>
       <c r="P59" t="inlineStr">
@@ -3534,6 +3605,7 @@
           <t>Ci Siamo</t>
         </is>
       </c>
+      <c r="Q59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -3568,22 +3640,15 @@
       <c r="J60" t="n">
         <v>448</v>
       </c>
-      <c r="K60" t="n">
-        <v>4.323</v>
-      </c>
-      <c r="L60" t="n">
-        <v>90.8</v>
-      </c>
-      <c r="M60" t="n">
-        <v>4.449</v>
-      </c>
-      <c r="N60" t="n">
-        <v>77.8</v>
-      </c>
       <c r="O60" t="inlineStr"/>
       <c r="P60" t="inlineStr">
         <is>
           <t>Tarallucci e Vino NoMad</t>
+        </is>
+      </c>
+      <c r="Q60" t="inlineStr">
+        <is>
+          <t>Google rating 4.6 excluded — Google returned 'Tarallucci e Vino NoMad', whose name similarity to 'Bar Tulia' is 0.36 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -3624,13 +3689,13 @@
         <v>4.187</v>
       </c>
       <c r="L61" t="n">
-        <v>77.8</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="M61" t="n">
         <v>4.079</v>
       </c>
       <c r="N61" t="n">
-        <v>31.4</v>
+        <v>32.9</v>
       </c>
       <c r="O61" t="inlineStr"/>
       <c r="P61" t="inlineStr">
@@ -3638,6 +3703,7 @@
           <t>Santi</t>
         </is>
       </c>
+      <c r="Q61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -3676,13 +3742,13 @@
         <v>4.07</v>
       </c>
       <c r="L62" t="n">
-        <v>56.9</v>
+        <v>59.2</v>
       </c>
       <c r="M62" t="n">
         <v>4.461</v>
       </c>
       <c r="N62" t="n">
-        <v>80.40000000000001</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="O62" t="inlineStr"/>
       <c r="P62" t="inlineStr">
@@ -3690,6 +3756,7 @@
           <t>Ribalta</t>
         </is>
       </c>
+      <c r="Q62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -3728,13 +3795,13 @@
         <v>4.127</v>
       </c>
       <c r="L63" t="n">
-        <v>67.3</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="M63" t="n">
         <v>4.523</v>
       </c>
       <c r="N63" t="n">
-        <v>85.59999999999999</v>
+        <v>86.2</v>
       </c>
       <c r="O63" t="inlineStr"/>
       <c r="P63" t="inlineStr">
@@ -3742,6 +3809,7 @@
           <t>Don Antonio</t>
         </is>
       </c>
+      <c r="Q63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -3780,13 +3848,13 @@
         <v>4.138</v>
       </c>
       <c r="L64" t="n">
-        <v>71.2</v>
+        <v>73</v>
       </c>
       <c r="M64" t="n">
         <v>4.535</v>
       </c>
       <c r="N64" t="n">
-        <v>86.90000000000001</v>
+        <v>87.5</v>
       </c>
       <c r="O64" t="inlineStr"/>
       <c r="P64" t="inlineStr">
@@ -3794,6 +3862,7 @@
           <t>Kesté Pizza e Vino</t>
         </is>
       </c>
+      <c r="Q64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -3832,13 +3901,13 @@
         <v>4.137</v>
       </c>
       <c r="L65" t="n">
-        <v>70.59999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="M65" t="n">
         <v>4.03</v>
       </c>
       <c r="N65" t="n">
-        <v>22.9</v>
+        <v>25</v>
       </c>
       <c r="O65" t="inlineStr"/>
       <c r="P65" t="inlineStr">
@@ -3846,6 +3915,7 @@
           <t>Rao's</t>
         </is>
       </c>
+      <c r="Q65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -3898,6 +3968,7 @@
           <t>Elio's</t>
         </is>
       </c>
+      <c r="Q66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -3933,21 +4004,26 @@
         <v>1002</v>
       </c>
       <c r="K67" t="n">
-        <v>3.948</v>
+        <v>3.856</v>
       </c>
       <c r="L67" t="n">
-        <v>23.5</v>
+        <v>11.2</v>
       </c>
       <c r="M67" t="n">
-        <v>4.063</v>
+        <v>3.969</v>
       </c>
       <c r="N67" t="n">
-        <v>28.1</v>
+        <v>17.8</v>
       </c>
       <c r="O67" t="inlineStr"/>
       <c r="P67" t="inlineStr">
         <is>
           <t>Sant Ambroeus Madison</t>
+        </is>
+      </c>
+      <c r="Q67" t="inlineStr">
+        <is>
+          <t>Google rating 4.3 excluded — Google returned 'Sant Ambroeus Madison', whose name similarity to 'Sant Ambroeus UES' is 0.76 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -3988,13 +4064,13 @@
         <v>4.251</v>
       </c>
       <c r="L68" t="n">
-        <v>81</v>
+        <v>82.2</v>
       </c>
       <c r="M68" t="n">
         <v>4.375</v>
       </c>
       <c r="N68" t="n">
-        <v>68.59999999999999</v>
+        <v>69.7</v>
       </c>
       <c r="O68" t="inlineStr"/>
       <c r="P68" t="inlineStr">
@@ -4002,6 +4078,7 @@
           <t>Sempre Oggi</t>
         </is>
       </c>
+      <c r="Q68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -4040,13 +4117,13 @@
         <v>3.781</v>
       </c>
       <c r="L69" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="M69" t="n">
         <v>3.891</v>
       </c>
       <c r="N69" t="n">
-        <v>10.5</v>
+        <v>11.2</v>
       </c>
       <c r="O69" t="inlineStr"/>
       <c r="P69" t="inlineStr">
@@ -4054,6 +4131,7 @@
           <t>Cafe Fiorello</t>
         </is>
       </c>
+      <c r="Q69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -4092,13 +4170,13 @@
         <v>3.932</v>
       </c>
       <c r="L70" t="n">
-        <v>20.9</v>
+        <v>24.3</v>
       </c>
       <c r="M70" t="n">
         <v>3.831</v>
       </c>
       <c r="N70" t="n">
-        <v>7.2</v>
+        <v>7.9</v>
       </c>
       <c r="O70" t="inlineStr"/>
       <c r="P70" t="inlineStr">
@@ -4106,6 +4184,7 @@
           <t>Lincoln Ristorante</t>
         </is>
       </c>
+      <c r="Q70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -4150,7 +4229,7 @@
         <v>4.043</v>
       </c>
       <c r="N71" t="n">
-        <v>25.5</v>
+        <v>27.6</v>
       </c>
       <c r="O71" t="inlineStr"/>
       <c r="P71" t="inlineStr">
@@ -4158,6 +4237,7 @@
           <t>Tarallucci e Vino Upper West Side</t>
         </is>
       </c>
+      <c r="Q71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -4196,13 +4276,13 @@
         <v>4.077</v>
       </c>
       <c r="L72" t="n">
-        <v>58.8</v>
+        <v>61.2</v>
       </c>
       <c r="M72" t="n">
         <v>4.468</v>
       </c>
       <c r="N72" t="n">
-        <v>81.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="O72" t="inlineStr"/>
       <c r="P72" t="inlineStr">
@@ -4210,6 +4290,7 @@
           <t>Patsy's Pizzeria</t>
         </is>
       </c>
+      <c r="Q72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -4245,21 +4326,26 @@
         <v>1576</v>
       </c>
       <c r="K73" t="n">
-        <v>4.105</v>
+        <v>3.895</v>
       </c>
       <c r="L73" t="n">
-        <v>63.4</v>
+        <v>15.8</v>
       </c>
       <c r="M73" t="n">
-        <v>4.499</v>
+        <v>4.269</v>
       </c>
       <c r="N73" t="n">
-        <v>84.3</v>
+        <v>60.5</v>
       </c>
       <c r="O73" t="inlineStr"/>
       <c r="P73" t="inlineStr">
         <is>
           <t>Sottocasa Pizzeria Harlem</t>
+        </is>
+      </c>
+      <c r="Q73" t="inlineStr">
+        <is>
+          <t>Google rating 4.7 excluded — Google returned 'Sottocasa Pizzeria Harlem', whose name similarity to 'Sottocasa Harlem' is 0.79 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -4300,13 +4386,13 @@
         <v>4.05</v>
       </c>
       <c r="L74" t="n">
-        <v>49.7</v>
+        <v>52.6</v>
       </c>
       <c r="M74" t="n">
         <v>4.071</v>
       </c>
       <c r="N74" t="n">
-        <v>30.1</v>
+        <v>31.6</v>
       </c>
       <c r="O74" t="inlineStr"/>
       <c r="P74" t="inlineStr">
@@ -4314,6 +4400,7 @@
           <t>Lilia</t>
         </is>
       </c>
+      <c r="Q74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -4352,13 +4439,13 @@
         <v>4.058</v>
       </c>
       <c r="L75" t="n">
-        <v>52.9</v>
+        <v>55.9</v>
       </c>
       <c r="M75" t="n">
         <v>4.124</v>
       </c>
       <c r="N75" t="n">
-        <v>38.6</v>
+        <v>40.1</v>
       </c>
       <c r="O75" t="inlineStr"/>
       <c r="P75" t="inlineStr">
@@ -4366,6 +4453,7 @@
           <t>Misi</t>
         </is>
       </c>
+      <c r="Q75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -4404,13 +4492,13 @@
         <v>3.968</v>
       </c>
       <c r="L76" t="n">
-        <v>26.8</v>
+        <v>29.6</v>
       </c>
       <c r="M76" t="n">
         <v>3.968</v>
       </c>
       <c r="N76" t="n">
-        <v>16.3</v>
+        <v>16.4</v>
       </c>
       <c r="O76" t="inlineStr"/>
       <c r="P76" t="inlineStr">
@@ -4418,6 +4506,7 @@
           <t>I Cavallini</t>
         </is>
       </c>
+      <c r="Q76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -4456,13 +4545,13 @@
         <v>4.051</v>
       </c>
       <c r="L77" t="n">
-        <v>50.3</v>
+        <v>53.3</v>
       </c>
       <c r="M77" t="n">
         <v>4.17</v>
       </c>
       <c r="N77" t="n">
-        <v>45.8</v>
+        <v>47.4</v>
       </c>
       <c r="O77" t="inlineStr"/>
       <c r="P77" t="inlineStr">
@@ -4470,6 +4559,7 @@
           <t>Bamonte's</t>
         </is>
       </c>
+      <c r="Q77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -4508,13 +4598,13 @@
         <v>4.223</v>
       </c>
       <c r="L78" t="n">
-        <v>79.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="M78" t="n">
         <v>4.346</v>
       </c>
       <c r="N78" t="n">
-        <v>66</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="O78" t="inlineStr"/>
       <c r="P78" t="inlineStr">
@@ -4522,6 +4612,7 @@
           <t>Aurora Brooklyn</t>
         </is>
       </c>
+      <c r="Q78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -4560,13 +4651,13 @@
         <v>3.858</v>
       </c>
       <c r="L79" t="n">
-        <v>10.5</v>
+        <v>11.8</v>
       </c>
       <c r="M79" t="n">
         <v>3.971</v>
       </c>
       <c r="N79" t="n">
-        <v>17.6</v>
+        <v>18.4</v>
       </c>
       <c r="O79" t="inlineStr"/>
       <c r="P79" t="inlineStr">
@@ -4574,6 +4665,7 @@
           <t>Fabbrica | The Factory</t>
         </is>
       </c>
+      <c r="Q79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -4612,13 +4704,13 @@
         <v>3.91</v>
       </c>
       <c r="L80" t="n">
-        <v>16.3</v>
+        <v>19.7</v>
       </c>
       <c r="M80" t="n">
         <v>4.285</v>
       </c>
       <c r="N80" t="n">
-        <v>61.4</v>
+        <v>62.5</v>
       </c>
       <c r="O80" t="inlineStr"/>
       <c r="P80" t="inlineStr">
@@ -4626,6 +4718,7 @@
           <t>Sauced</t>
         </is>
       </c>
+      <c r="Q80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -4664,13 +4757,13 @@
         <v>4.14</v>
       </c>
       <c r="L81" t="n">
-        <v>72.5</v>
+        <v>74.3</v>
       </c>
       <c r="M81" t="n">
         <v>4.537</v>
       </c>
       <c r="N81" t="n">
-        <v>87.59999999999999</v>
+        <v>88.2</v>
       </c>
       <c r="O81" t="inlineStr"/>
       <c r="P81" t="inlineStr">
@@ -4678,6 +4771,7 @@
           <t>Sottocasa</t>
         </is>
       </c>
+      <c r="Q81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -4716,13 +4810,13 @@
         <v>4.108</v>
       </c>
       <c r="L82" t="n">
-        <v>64.7</v>
+        <v>66.40000000000001</v>
       </c>
       <c r="M82" t="n">
         <v>4.288</v>
       </c>
       <c r="N82" t="n">
-        <v>62.1</v>
+        <v>63.2</v>
       </c>
       <c r="O82" t="inlineStr"/>
       <c r="P82" t="inlineStr">
@@ -4730,6 +4824,7 @@
           <t>Frankies 457 Spuntino</t>
         </is>
       </c>
+      <c r="Q82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -4768,13 +4863,13 @@
         <v>4.027</v>
       </c>
       <c r="L83" t="n">
-        <v>43.1</v>
+        <v>46.1</v>
       </c>
       <c r="M83" t="n">
         <v>4.78</v>
       </c>
       <c r="N83" t="n">
-        <v>96.09999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="O83" t="inlineStr"/>
       <c r="P83" t="inlineStr">
@@ -4782,6 +4877,7 @@
           <t>F&amp;F Pizzeria</t>
         </is>
       </c>
+      <c r="Q83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -4820,13 +4916,13 @@
         <v>4.057</v>
       </c>
       <c r="L84" t="n">
-        <v>51.6</v>
+        <v>54.6</v>
       </c>
       <c r="M84" t="n">
         <v>4.175</v>
       </c>
       <c r="N84" t="n">
-        <v>47.1</v>
+        <v>48.7</v>
       </c>
       <c r="O84" t="inlineStr"/>
       <c r="P84" t="inlineStr">
@@ -4834,6 +4930,7 @@
           <t>Cafe Spaghetti</t>
         </is>
       </c>
+      <c r="Q84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -4872,13 +4969,13 @@
         <v>4.356</v>
       </c>
       <c r="L85" t="n">
-        <v>94.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="M85" t="n">
         <v>4.484</v>
       </c>
       <c r="N85" t="n">
-        <v>83.7</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="O85" t="inlineStr"/>
       <c r="P85" t="inlineStr">
@@ -4886,6 +4983,7 @@
           <t>Cremini's</t>
         </is>
       </c>
+      <c r="Q85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -4924,13 +5022,13 @@
         <v>4.306</v>
       </c>
       <c r="L86" t="n">
-        <v>88.90000000000001</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="M86" t="n">
         <v>4.432</v>
       </c>
       <c r="N86" t="n">
-        <v>75.2</v>
+        <v>77</v>
       </c>
       <c r="O86" t="inlineStr"/>
       <c r="P86" t="inlineStr">
@@ -4938,6 +5036,7 @@
           <t>Lucali</t>
         </is>
       </c>
+      <c r="Q86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -4976,13 +5075,13 @@
         <v>4.013</v>
       </c>
       <c r="L87" t="n">
-        <v>37.9</v>
+        <v>40.8</v>
       </c>
       <c r="M87" t="n">
         <v>4.13</v>
       </c>
       <c r="N87" t="n">
-        <v>41.2</v>
+        <v>42.8</v>
       </c>
       <c r="O87" t="inlineStr"/>
       <c r="P87" t="inlineStr">
@@ -4990,6 +5089,7 @@
           <t>Marco Polo</t>
         </is>
       </c>
+      <c r="Q87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5028,13 +5128,13 @@
         <v>4.016</v>
       </c>
       <c r="L88" t="n">
-        <v>39.2</v>
+        <v>42.1</v>
       </c>
       <c r="M88" t="n">
         <v>4.767</v>
       </c>
       <c r="N88" t="n">
-        <v>94.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="O88" t="inlineStr"/>
       <c r="P88" t="inlineStr">
@@ -5042,6 +5142,7 @@
           <t>Bar Ferdinando</t>
         </is>
       </c>
+      <c r="Q88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5080,13 +5181,13 @@
         <v>4.021</v>
       </c>
       <c r="L89" t="n">
-        <v>41.2</v>
+        <v>44.1</v>
       </c>
       <c r="M89" t="n">
         <v>4.138</v>
       </c>
       <c r="N89" t="n">
-        <v>41.8</v>
+        <v>43.4</v>
       </c>
       <c r="O89" t="inlineStr"/>
       <c r="P89" t="inlineStr">
@@ -5094,6 +5195,7 @@
           <t>Noodle Pudding</t>
         </is>
       </c>
+      <c r="Q89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -5132,13 +5234,13 @@
         <v>3.927</v>
       </c>
       <c r="L90" t="n">
-        <v>18.3</v>
+        <v>21.7</v>
       </c>
       <c r="M90" t="n">
         <v>4.041</v>
       </c>
       <c r="N90" t="n">
-        <v>24.8</v>
+        <v>27</v>
       </c>
       <c r="O90" t="inlineStr"/>
       <c r="P90" t="inlineStr">
@@ -5146,6 +5248,7 @@
           <t>River Deli</t>
         </is>
       </c>
+      <c r="Q90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5184,13 +5287,13 @@
         <v>4.057</v>
       </c>
       <c r="L91" t="n">
-        <v>52.3</v>
+        <v>55.3</v>
       </c>
       <c r="M91" t="n">
         <v>4.176</v>
       </c>
       <c r="N91" t="n">
-        <v>47.7</v>
+        <v>49.3</v>
       </c>
       <c r="O91" t="inlineStr"/>
       <c r="P91" t="inlineStr">
@@ -5198,6 +5301,7 @@
           <t>al di là Trattoria</t>
         </is>
       </c>
+      <c r="Q91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5250,6 +5354,7 @@
           <t>Lillo Cucina Italiana</t>
         </is>
       </c>
+      <c r="Q92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5288,13 +5393,13 @@
         <v>4.066</v>
       </c>
       <c r="L93" t="n">
-        <v>54.9</v>
+        <v>57.2</v>
       </c>
       <c r="M93" t="n">
         <v>4.456</v>
       </c>
       <c r="N93" t="n">
-        <v>78.40000000000001</v>
+        <v>79.59999999999999</v>
       </c>
       <c r="O93" t="inlineStr"/>
       <c r="P93" t="inlineStr">
@@ -5302,6 +5407,7 @@
           <t>Roberta's</t>
         </is>
       </c>
+      <c r="Q93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -5340,13 +5446,13 @@
         <v>4.296</v>
       </c>
       <c r="L94" t="n">
-        <v>86.3</v>
+        <v>87.5</v>
       </c>
       <c r="M94" t="n">
         <v>4.421</v>
       </c>
       <c r="N94" t="n">
-        <v>74.5</v>
+        <v>76.3</v>
       </c>
       <c r="O94" t="inlineStr"/>
       <c r="P94" t="inlineStr">
@@ -5354,6 +5460,7 @@
           <t>Faro</t>
         </is>
       </c>
+      <c r="Q94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -5392,13 +5499,13 @@
         <v>4.072</v>
       </c>
       <c r="L95" t="n">
-        <v>58.2</v>
+        <v>60.5</v>
       </c>
       <c r="M95" t="n">
         <v>4.463</v>
       </c>
       <c r="N95" t="n">
-        <v>81</v>
+        <v>82.2</v>
       </c>
       <c r="O95" t="inlineStr"/>
       <c r="P95" t="inlineStr">
@@ -5406,6 +5513,7 @@
           <t>Saraghina Pizzeria</t>
         </is>
       </c>
+      <c r="Q95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5444,13 +5552,13 @@
         <v>3.973</v>
       </c>
       <c r="L96" t="n">
-        <v>28.8</v>
+        <v>31.6</v>
       </c>
       <c r="M96" t="n">
         <v>3.87</v>
       </c>
       <c r="N96" t="n">
-        <v>7.8</v>
+        <v>8.6</v>
       </c>
       <c r="O96" t="inlineStr"/>
       <c r="P96" t="inlineStr">
@@ -5458,6 +5566,7 @@
           <t>Gargiulo's</t>
         </is>
       </c>
+      <c r="Q96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5496,13 +5605,13 @@
         <v>4.334</v>
       </c>
       <c r="L97" t="n">
-        <v>92.8</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="M97" t="n">
         <v>4.749</v>
       </c>
       <c r="N97" t="n">
-        <v>94.09999999999999</v>
+        <v>94.7</v>
       </c>
       <c r="O97" t="inlineStr"/>
       <c r="P97" t="inlineStr">
@@ -5510,6 +5619,7 @@
           <t>L&amp;B Spumoni Gardens</t>
         </is>
       </c>
+      <c r="Q97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5548,13 +5658,13 @@
         <v>3.925</v>
       </c>
       <c r="L98" t="n">
-        <v>17.6</v>
+        <v>21.1</v>
       </c>
       <c r="M98" t="n">
         <v>4.039</v>
       </c>
       <c r="N98" t="n">
-        <v>24.2</v>
+        <v>26.3</v>
       </c>
       <c r="O98" t="inlineStr"/>
       <c r="P98" t="inlineStr">
@@ -5562,6 +5672,7 @@
           <t>Tommaso</t>
         </is>
       </c>
+      <c r="Q98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5600,13 +5711,13 @@
         <v>4.292</v>
       </c>
       <c r="L99" t="n">
-        <v>85.59999999999999</v>
+        <v>86.8</v>
       </c>
       <c r="M99" t="n">
         <v>4.417</v>
       </c>
       <c r="N99" t="n">
-        <v>73.2</v>
+        <v>75</v>
       </c>
       <c r="O99" t="inlineStr"/>
       <c r="P99" t="inlineStr">
@@ -5614,6 +5725,7 @@
           <t>Il Colosseo Ristorante | Brooklyn</t>
         </is>
       </c>
+      <c r="Q99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5652,13 +5764,13 @@
         <v>4.089</v>
       </c>
       <c r="L100" t="n">
-        <v>61.4</v>
+        <v>63.8</v>
       </c>
       <c r="M100" t="n">
         <v>4.209</v>
       </c>
       <c r="N100" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="O100" t="inlineStr"/>
       <c r="P100" t="inlineStr">
@@ -5666,6 +5778,7 @@
           <t>Ortobello's</t>
         </is>
       </c>
+      <c r="Q100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5710,7 +5823,7 @@
         <v>4.12</v>
       </c>
       <c r="N101" t="n">
-        <v>36.6</v>
+        <v>38.2</v>
       </c>
       <c r="O101" t="inlineStr"/>
       <c r="P101" t="inlineStr">
@@ -5718,6 +5831,7 @@
           <t>Randazzo's Clam Bar</t>
         </is>
       </c>
+      <c r="Q101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5756,13 +5870,13 @@
         <v>4.135</v>
       </c>
       <c r="L102" t="n">
-        <v>69.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="M102" t="n">
         <v>4.256</v>
       </c>
       <c r="N102" t="n">
-        <v>56.9</v>
+        <v>58.6</v>
       </c>
       <c r="O102" t="inlineStr"/>
       <c r="P102" t="inlineStr">
@@ -5770,6 +5884,7 @@
           <t>Michael’s</t>
         </is>
       </c>
+      <c r="Q102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5808,13 +5923,13 @@
         <v>4.069</v>
       </c>
       <c r="L103" t="n">
-        <v>56.2</v>
+        <v>58.6</v>
       </c>
       <c r="M103" t="n">
         <v>4.46</v>
       </c>
       <c r="N103" t="n">
-        <v>79.7</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="O103" t="inlineStr"/>
       <c r="P103" t="inlineStr">
@@ -5822,6 +5937,7 @@
           <t>Di Fara Pizza</t>
         </is>
       </c>
+      <c r="Q103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5874,6 +5990,7 @@
           <t>Ponte Vecchio</t>
         </is>
       </c>
+      <c r="Q104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -5912,13 +6029,13 @@
         <v>4.104</v>
       </c>
       <c r="L105" t="n">
-        <v>62.7</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="M105" t="n">
         <v>4.224</v>
       </c>
       <c r="N105" t="n">
-        <v>51.6</v>
+        <v>52.6</v>
       </c>
       <c r="O105" t="inlineStr"/>
       <c r="P105" t="inlineStr">
@@ -5926,6 +6043,7 @@
           <t>Gino's</t>
         </is>
       </c>
+      <c r="Q105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -5964,13 +6082,13 @@
         <v>4.046</v>
       </c>
       <c r="L106" t="n">
-        <v>47.7</v>
+        <v>50.7</v>
       </c>
       <c r="M106" t="n">
         <v>4.165</v>
       </c>
       <c r="N106" t="n">
-        <v>44.4</v>
+        <v>46.1</v>
       </c>
       <c r="O106" t="inlineStr"/>
       <c r="P106" t="inlineStr">
@@ -5978,6 +6096,7 @@
           <t>Positano</t>
         </is>
       </c>
+      <c r="Q106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -6016,13 +6135,13 @@
         <v>4.044</v>
       </c>
       <c r="L107" t="n">
-        <v>46.4</v>
+        <v>49.3</v>
       </c>
       <c r="M107" t="n">
         <v>4.432</v>
       </c>
       <c r="N107" t="n">
-        <v>75.8</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="O107" t="inlineStr"/>
       <c r="P107" t="inlineStr">
@@ -6030,6 +6149,7 @@
           <t>Lombardo’s of Bay Ridge</t>
         </is>
       </c>
+      <c r="Q107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -6074,7 +6194,7 @@
         <v>3.782</v>
       </c>
       <c r="N108" t="n">
-        <v>3.9</v>
+        <v>4.6</v>
       </c>
       <c r="O108" t="inlineStr"/>
       <c r="P108" t="inlineStr">
@@ -6082,6 +6202,7 @@
           <t>Greenhouse Cafe</t>
         </is>
       </c>
+      <c r="Q108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -6120,13 +6241,13 @@
         <v>3.985</v>
       </c>
       <c r="L109" t="n">
-        <v>32</v>
+        <v>34.9</v>
       </c>
       <c r="M109" t="n">
         <v>4.102</v>
       </c>
       <c r="N109" t="n">
-        <v>35.9</v>
+        <v>37.5</v>
       </c>
       <c r="O109" t="inlineStr"/>
       <c r="P109" t="inlineStr">
@@ -6134,6 +6255,7 @@
           <t>La Nonna Ristorante &amp; Bar - Williamsburg, Brooklyn</t>
         </is>
       </c>
+      <c r="Q109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -6172,13 +6294,13 @@
         <v>4.124</v>
       </c>
       <c r="L110" t="n">
-        <v>66.7</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="M110" t="n">
         <v>4.244</v>
       </c>
       <c r="N110" t="n">
-        <v>54.2</v>
+        <v>55.3</v>
       </c>
       <c r="O110" t="inlineStr"/>
       <c r="P110" t="inlineStr">
@@ -6186,6 +6308,7 @@
           <t>LaRina Pastificio &amp; Vino</t>
         </is>
       </c>
+      <c r="Q110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -6224,13 +6347,13 @@
         <v>4.008</v>
       </c>
       <c r="L111" t="n">
-        <v>36.6</v>
+        <v>39.5</v>
       </c>
       <c r="M111" t="n">
         <v>4.125</v>
       </c>
       <c r="N111" t="n">
-        <v>39.2</v>
+        <v>40.8</v>
       </c>
       <c r="O111" t="inlineStr"/>
       <c r="P111" t="inlineStr">
@@ -6238,6 +6361,7 @@
           <t>Locanda Vini &amp; Olii</t>
         </is>
       </c>
+      <c r="Q111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -6276,13 +6400,13 @@
         <v>3.908</v>
       </c>
       <c r="L112" t="n">
-        <v>15.7</v>
+        <v>19.1</v>
       </c>
       <c r="M112" t="n">
         <v>3.807</v>
       </c>
       <c r="N112" t="n">
-        <v>5.9</v>
+        <v>6.6</v>
       </c>
       <c r="O112" t="inlineStr"/>
       <c r="P112" t="inlineStr">
@@ -6290,6 +6414,7 @@
           <t>Cecconi's DUMBO</t>
         </is>
       </c>
+      <c r="Q112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -6328,13 +6453,13 @@
         <v>4.302</v>
       </c>
       <c r="L113" t="n">
-        <v>87.59999999999999</v>
+        <v>88.8</v>
       </c>
       <c r="M113" t="n">
         <v>4.715</v>
       </c>
       <c r="N113" t="n">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="O113" t="inlineStr"/>
       <c r="P113" t="inlineStr">
@@ -6342,6 +6467,7 @@
           <t>Juliana’s</t>
         </is>
       </c>
+      <c r="Q113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -6380,13 +6506,13 @@
         <v>3.725</v>
       </c>
       <c r="L114" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
       <c r="M114" t="n">
         <v>4.082</v>
       </c>
       <c r="N114" t="n">
-        <v>33.3</v>
+        <v>34.9</v>
       </c>
       <c r="O114" t="inlineStr"/>
       <c r="P114" t="inlineStr">
@@ -6394,6 +6520,7 @@
           <t>Grimaldi's Pizzeria</t>
         </is>
       </c>
+      <c r="Q114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -6432,13 +6559,13 @@
         <v>4.085</v>
       </c>
       <c r="L115" t="n">
-        <v>60.1</v>
+        <v>62.5</v>
       </c>
       <c r="M115" t="n">
         <v>4.204</v>
       </c>
       <c r="N115" t="n">
-        <v>49.7</v>
+        <v>50.7</v>
       </c>
       <c r="O115" t="inlineStr"/>
       <c r="P115" t="inlineStr">
@@ -6446,6 +6573,7 @@
           <t>Park Side Restaurant</t>
         </is>
       </c>
+      <c r="Q115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -6481,21 +6609,26 @@
         <v>1493</v>
       </c>
       <c r="K116" t="n">
-        <v>4.157</v>
+        <v>3.896</v>
       </c>
       <c r="L116" t="n">
-        <v>74.5</v>
+        <v>17.8</v>
       </c>
       <c r="M116" t="n">
-        <v>4.278</v>
+        <v>4.01</v>
       </c>
       <c r="N116" t="n">
-        <v>60.1</v>
+        <v>23.7</v>
       </c>
       <c r="O116" t="inlineStr"/>
       <c r="P116" t="inlineStr">
         <is>
           <t>L’incontro by Rocco</t>
+        </is>
+      </c>
+      <c r="Q116" t="inlineStr">
+        <is>
+          <t>Google rating 4.7 excluded — Google returned 'L’incontro by Rocco', whose name similarity to "Trattoria L'Incontro" is 0.53 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -6536,13 +6669,13 @@
         <v>4.086</v>
       </c>
       <c r="L117" t="n">
-        <v>60.8</v>
+        <v>63.2</v>
       </c>
       <c r="M117" t="n">
         <v>4.205</v>
       </c>
       <c r="N117" t="n">
-        <v>50.3</v>
+        <v>51.3</v>
       </c>
       <c r="O117" t="inlineStr"/>
       <c r="P117" t="inlineStr">
@@ -6550,6 +6683,7 @@
           <t>Don Peppe</t>
         </is>
       </c>
+      <c r="Q117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6588,13 +6722,13 @@
         <v>4.003</v>
       </c>
       <c r="L118" t="n">
-        <v>34</v>
+        <v>36.8</v>
       </c>
       <c r="M118" t="n">
         <v>4.12</v>
       </c>
       <c r="N118" t="n">
-        <v>37.3</v>
+        <v>38.8</v>
       </c>
       <c r="O118" t="inlineStr"/>
       <c r="P118" t="inlineStr">
@@ -6602,6 +6736,7 @@
           <t>Manducatis</t>
         </is>
       </c>
+      <c r="Q118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6640,13 +6775,13 @@
         <v>3.986</v>
       </c>
       <c r="L119" t="n">
-        <v>33.3</v>
+        <v>36.2</v>
       </c>
       <c r="M119" t="n">
         <v>4.369</v>
       </c>
       <c r="N119" t="n">
-        <v>68</v>
+        <v>69.09999999999999</v>
       </c>
       <c r="O119" t="inlineStr"/>
       <c r="P119" t="inlineStr">
@@ -6654,6 +6789,7 @@
           <t>Manducatis Rustica VIG</t>
         </is>
       </c>
+      <c r="Q119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -6692,13 +6828,13 @@
         <v>4.078</v>
       </c>
       <c r="L120" t="n">
-        <v>59.5</v>
+        <v>61.8</v>
       </c>
       <c r="M120" t="n">
         <v>4.469</v>
       </c>
       <c r="N120" t="n">
-        <v>82.40000000000001</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="O120" t="inlineStr"/>
       <c r="P120" t="inlineStr">
@@ -6706,6 +6842,7 @@
           <t>Vesta Trattoria &amp; Wine Bar</t>
         </is>
       </c>
+      <c r="Q120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -6744,13 +6881,13 @@
         <v>4.328</v>
       </c>
       <c r="L121" t="n">
-        <v>92.2</v>
+        <v>92.8</v>
       </c>
       <c r="M121" t="n">
         <v>4.743</v>
       </c>
       <c r="N121" t="n">
-        <v>93.5</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="O121" t="inlineStr"/>
       <c r="P121" t="inlineStr">
@@ -6758,6 +6895,7 @@
           <t>Il Bambino</t>
         </is>
       </c>
+      <c r="Q121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6796,13 +6934,13 @@
         <v>4.382</v>
       </c>
       <c r="L122" t="n">
-        <v>95.40000000000001</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="M122" t="n">
         <v>4.509</v>
       </c>
       <c r="N122" t="n">
-        <v>85</v>
+        <v>85.5</v>
       </c>
       <c r="O122" t="inlineStr"/>
       <c r="P122" t="inlineStr">
@@ -6810,6 +6948,7 @@
           <t>VITE vinosteria</t>
         </is>
       </c>
+      <c r="Q122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6848,13 +6987,13 @@
         <v>4.28</v>
       </c>
       <c r="L123" t="n">
-        <v>85</v>
+        <v>86.2</v>
       </c>
       <c r="M123" t="n">
         <v>4.405</v>
       </c>
       <c r="N123" t="n">
-        <v>71.2</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="O123" t="inlineStr"/>
       <c r="P123" t="inlineStr">
@@ -6862,6 +7001,7 @@
           <t>Via Trenta Osteria &amp; Wine Bar</t>
         </is>
       </c>
+      <c r="Q123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -6900,13 +7040,13 @@
         <v>4.159</v>
       </c>
       <c r="L124" t="n">
-        <v>75.2</v>
+        <v>76.3</v>
       </c>
       <c r="M124" t="n">
         <v>4.28</v>
       </c>
       <c r="N124" t="n">
-        <v>60.8</v>
+        <v>61.8</v>
       </c>
       <c r="O124" t="inlineStr"/>
       <c r="P124" t="inlineStr">
@@ -6914,6 +7054,7 @@
           <t>VIA VAI</t>
         </is>
       </c>
+      <c r="Q124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -6952,13 +7093,13 @@
         <v>4.069</v>
       </c>
       <c r="L125" t="n">
-        <v>55.6</v>
+        <v>57.9</v>
       </c>
       <c r="M125" t="n">
         <v>4.459</v>
       </c>
       <c r="N125" t="n">
-        <v>79.09999999999999</v>
+        <v>80.3</v>
       </c>
       <c r="O125" t="inlineStr"/>
       <c r="P125" t="inlineStr">
@@ -6966,6 +7107,7 @@
           <t>Sac's Place</t>
         </is>
       </c>
+      <c r="Q125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -7004,13 +7146,13 @@
         <v>4.047</v>
       </c>
       <c r="L126" t="n">
-        <v>48.4</v>
+        <v>51.3</v>
       </c>
       <c r="M126" t="n">
         <v>3.942</v>
       </c>
       <c r="N126" t="n">
-        <v>14.4</v>
+        <v>14.5</v>
       </c>
       <c r="O126" t="inlineStr"/>
       <c r="P126" t="inlineStr">
@@ -7018,6 +7160,7 @@
           <t>Rialto Ristorante</t>
         </is>
       </c>
+      <c r="Q126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -7056,13 +7199,13 @@
         <v>4.256</v>
       </c>
       <c r="L127" t="n">
-        <v>81.7</v>
+        <v>82.90000000000001</v>
       </c>
       <c r="M127" t="n">
         <v>4.38</v>
       </c>
       <c r="N127" t="n">
-        <v>69.3</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="O127" t="inlineStr"/>
       <c r="P127" t="inlineStr">
@@ -7070,6 +7213,7 @@
           <t>Il Poeta</t>
         </is>
       </c>
+      <c r="Q127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -7108,13 +7252,13 @@
         <v>4.108</v>
       </c>
       <c r="L128" t="n">
-        <v>64.09999999999999</v>
+        <v>65.8</v>
       </c>
       <c r="M128" t="n">
         <v>4.227</v>
       </c>
       <c r="N128" t="n">
-        <v>52.3</v>
+        <v>53.3</v>
       </c>
       <c r="O128" t="inlineStr"/>
       <c r="P128" t="inlineStr">
@@ -7122,6 +7266,7 @@
           <t>Bruno</t>
         </is>
       </c>
+      <c r="Q128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -7157,21 +7302,26 @@
         <v>1799</v>
       </c>
       <c r="K129" t="n">
-        <v>4.38</v>
+        <v>4.368</v>
       </c>
       <c r="L129" t="n">
-        <v>94.8</v>
+        <v>95.40000000000001</v>
       </c>
       <c r="M129" t="n">
-        <v>4.267</v>
+        <v>4.255</v>
       </c>
       <c r="N129" t="n">
-        <v>58.8</v>
+        <v>57.2</v>
       </c>
       <c r="O129" t="inlineStr"/>
       <c r="P129" t="inlineStr">
         <is>
           <t>Vetro Restaurant &amp; Lounge</t>
+        </is>
+      </c>
+      <c r="Q129" t="inlineStr">
+        <is>
+          <t>Google rating 4.6 excluded — Google returned 'Vetro Restaurant &amp; Lounge', whose name similarity to "Vetro by Russo's on the Bay" is 0.48 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -7212,13 +7362,13 @@
         <v>4.048</v>
       </c>
       <c r="L130" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="M130" t="n">
         <v>4.436</v>
       </c>
       <c r="N130" t="n">
-        <v>76.5</v>
+        <v>78.3</v>
       </c>
       <c r="O130" t="inlineStr"/>
       <c r="P130" t="inlineStr">
@@ -7226,6 +7376,7 @@
           <t>Lenny's Clam Bar</t>
         </is>
       </c>
+      <c r="Q130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -7264,13 +7415,13 @@
         <v>3.945</v>
       </c>
       <c r="L131" t="n">
-        <v>22.9</v>
+        <v>26.3</v>
       </c>
       <c r="M131" t="n">
         <v>4.06</v>
       </c>
       <c r="N131" t="n">
-        <v>27.5</v>
+        <v>29.6</v>
       </c>
       <c r="O131" t="inlineStr"/>
       <c r="P131" t="inlineStr">
@@ -7278,6 +7429,7 @@
           <t>Matteo's of Howard Beach</t>
         </is>
       </c>
+      <c r="Q131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -7316,13 +7468,13 @@
         <v>4.02</v>
       </c>
       <c r="L132" t="n">
-        <v>40.5</v>
+        <v>43.4</v>
       </c>
       <c r="M132" t="n">
         <v>4.406</v>
       </c>
       <c r="N132" t="n">
-        <v>71.90000000000001</v>
+        <v>73</v>
       </c>
       <c r="O132" t="inlineStr"/>
       <c r="P132" t="inlineStr">
@@ -7330,6 +7482,7 @@
           <t>Riviera Ristorante</t>
         </is>
       </c>
+      <c r="Q132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -7368,13 +7521,13 @@
         <v>3.976</v>
       </c>
       <c r="L133" t="n">
-        <v>30.1</v>
+        <v>32.9</v>
       </c>
       <c r="M133" t="n">
         <v>4.092</v>
       </c>
       <c r="N133" t="n">
-        <v>34.6</v>
+        <v>36.2</v>
       </c>
       <c r="O133" t="inlineStr"/>
       <c r="P133" t="inlineStr">
@@ -7382,6 +7535,7 @@
           <t>Il Bacco</t>
         </is>
       </c>
+      <c r="Q133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -7420,13 +7574,13 @@
         <v>3.97</v>
       </c>
       <c r="L134" t="n">
-        <v>27.5</v>
+        <v>30.3</v>
       </c>
       <c r="M134" t="n">
         <v>4.713</v>
       </c>
       <c r="N134" t="n">
-        <v>91.5</v>
+        <v>92.09999999999999</v>
       </c>
       <c r="O134" t="inlineStr"/>
       <c r="P134" t="inlineStr">
@@ -7434,6 +7588,7 @@
           <t>Rosa's Pizza</t>
         </is>
       </c>
+      <c r="Q134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -7472,13 +7627,13 @@
         <v>4.151</v>
       </c>
       <c r="L135" t="n">
-        <v>73.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="M135" t="n">
         <v>4.549</v>
       </c>
       <c r="N135" t="n">
-        <v>88.2</v>
+        <v>88.8</v>
       </c>
       <c r="O135" t="inlineStr"/>
       <c r="P135" t="inlineStr">
@@ -7486,6 +7641,7 @@
           <t>Il Nonno</t>
         </is>
       </c>
+      <c r="Q135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -7524,13 +7680,13 @@
         <v>4.27</v>
       </c>
       <c r="L136" t="n">
-        <v>83</v>
+        <v>84.2</v>
       </c>
       <c r="M136" t="n">
         <v>4.68</v>
       </c>
       <c r="N136" t="n">
-        <v>90.8</v>
+        <v>91.40000000000001</v>
       </c>
       <c r="O136" t="inlineStr"/>
       <c r="P136" t="inlineStr">
@@ -7538,6 +7694,7 @@
           <t>Sotto la Luna</t>
         </is>
       </c>
+      <c r="Q136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -7576,13 +7733,13 @@
         <v>4.133</v>
       </c>
       <c r="L137" t="n">
-        <v>68.59999999999999</v>
+        <v>70.40000000000001</v>
       </c>
       <c r="M137" t="n">
         <v>4.529</v>
       </c>
       <c r="N137" t="n">
-        <v>86.3</v>
+        <v>86.8</v>
       </c>
       <c r="O137" t="inlineStr"/>
       <c r="P137" t="inlineStr">
@@ -7590,6 +7747,7 @@
           <t>Macoletta</t>
         </is>
       </c>
+      <c r="Q137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -7628,13 +7786,13 @@
         <v>3.956</v>
       </c>
       <c r="L138" t="n">
-        <v>24.8</v>
+        <v>27.6</v>
       </c>
       <c r="M138" t="n">
         <v>4.336</v>
       </c>
       <c r="N138" t="n">
-        <v>64.7</v>
+        <v>65.8</v>
       </c>
       <c r="O138" t="inlineStr"/>
       <c r="P138" t="inlineStr">
@@ -7642,6 +7800,7 @@
           <t>Palermo</t>
         </is>
       </c>
+      <c r="Q138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -7680,13 +7839,13 @@
         <v>4.038</v>
       </c>
       <c r="L139" t="n">
-        <v>45.1</v>
+        <v>48</v>
       </c>
       <c r="M139" t="n">
         <v>4.156</v>
       </c>
       <c r="N139" t="n">
-        <v>43.1</v>
+        <v>44.7</v>
       </c>
       <c r="O139" t="inlineStr"/>
       <c r="P139" t="inlineStr">
@@ -7694,6 +7853,7 @@
           <t>Roberto's</t>
         </is>
       </c>
+      <c r="Q139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -7732,13 +7892,13 @@
         <v>4.028</v>
       </c>
       <c r="L140" t="n">
-        <v>43.8</v>
+        <v>46.7</v>
       </c>
       <c r="M140" t="n">
         <v>4.145</v>
       </c>
       <c r="N140" t="n">
-        <v>42.5</v>
+        <v>44.1</v>
       </c>
       <c r="O140" t="inlineStr"/>
       <c r="P140" t="inlineStr">
@@ -7746,6 +7906,7 @@
           <t>Dominick's</t>
         </is>
       </c>
+      <c r="Q140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -7784,13 +7945,13 @@
         <v>3.972</v>
       </c>
       <c r="L141" t="n">
-        <v>28.1</v>
+        <v>30.9</v>
       </c>
       <c r="M141" t="n">
         <v>4.088</v>
       </c>
       <c r="N141" t="n">
-        <v>34</v>
+        <v>35.5</v>
       </c>
       <c r="O141" t="inlineStr"/>
       <c r="P141" t="inlineStr">
@@ -7798,6 +7959,7 @@
           <t>Mario's Restaurant of Arthur Avenue</t>
         </is>
       </c>
+      <c r="Q141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -7833,21 +7995,26 @@
         <v>1579</v>
       </c>
       <c r="K142" t="n">
-        <v>4.064</v>
+        <v>3.889</v>
       </c>
       <c r="L142" t="n">
-        <v>53.6</v>
+        <v>15.1</v>
       </c>
       <c r="M142" t="n">
-        <v>4.183</v>
+        <v>4.003</v>
       </c>
       <c r="N142" t="n">
-        <v>48.4</v>
+        <v>21.7</v>
       </c>
       <c r="O142" t="inlineStr"/>
       <c r="P142" t="inlineStr">
         <is>
           <t>Zero Otto Nove Bronx</t>
+        </is>
+      </c>
+      <c r="Q142" t="inlineStr">
+        <is>
+          <t>Google rating 4.5 excluded — Google returned 'Zero Otto Nove Bronx', whose name similarity to 'Zero Otto Nove (Trattoria)' is 0.74 — below the 0.80 trust threshold</t>
         </is>
       </c>
     </row>
@@ -7888,13 +8055,13 @@
         <v>3.982</v>
       </c>
       <c r="L143" t="n">
-        <v>31.4</v>
+        <v>34.2</v>
       </c>
       <c r="M143" t="n">
         <v>4.364</v>
       </c>
       <c r="N143" t="n">
-        <v>67.3</v>
+        <v>68.40000000000001</v>
       </c>
       <c r="O143" t="inlineStr"/>
       <c r="P143" t="inlineStr">
@@ -7902,6 +8069,7 @@
           <t>Tra Di Noi</t>
         </is>
       </c>
+      <c r="Q143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -7940,13 +8108,13 @@
         <v>4.005</v>
       </c>
       <c r="L144" t="n">
-        <v>35.9</v>
+        <v>38.8</v>
       </c>
       <c r="M144" t="n">
         <v>4.389</v>
       </c>
       <c r="N144" t="n">
-        <v>69.90000000000001</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="O144" t="inlineStr"/>
       <c r="P144" t="inlineStr">
@@ -7954,6 +8122,7 @@
           <t>Enzo's of Arthur Avenue</t>
         </is>
       </c>
+      <c r="Q144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -8006,6 +8175,7 @@
           <t>Antonio's Trattoria</t>
         </is>
       </c>
+      <c r="Q145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -8044,13 +8214,13 @@
         <v>3.884</v>
       </c>
       <c r="L146" t="n">
-        <v>13.1</v>
+        <v>14.5</v>
       </c>
       <c r="M146" t="n">
         <v>3.997</v>
       </c>
       <c r="N146" t="n">
-        <v>20.3</v>
+        <v>21.1</v>
       </c>
       <c r="O146" t="inlineStr"/>
       <c r="P146" t="inlineStr">
@@ -8058,6 +8228,7 @@
           <t>Pasquale's Rigoletto</t>
         </is>
       </c>
+      <c r="Q146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -8096,13 +8267,13 @@
         <v>4.034</v>
       </c>
       <c r="L147" t="n">
-        <v>44.4</v>
+        <v>47.4</v>
       </c>
       <c r="M147" t="n">
         <v>4.421</v>
       </c>
       <c r="N147" t="n">
-        <v>73.90000000000001</v>
+        <v>75.7</v>
       </c>
       <c r="O147" t="inlineStr"/>
       <c r="P147" t="inlineStr">
@@ -8110,6 +8281,7 @@
           <t>Emilia's</t>
         </is>
       </c>
+      <c r="Q147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -8148,13 +8320,13 @@
         <v>3.883</v>
       </c>
       <c r="L148" t="n">
-        <v>12.4</v>
+        <v>13.8</v>
       </c>
       <c r="M148" t="n">
         <v>4.256</v>
       </c>
       <c r="N148" t="n">
-        <v>56.2</v>
+        <v>57.9</v>
       </c>
       <c r="O148" t="inlineStr"/>
       <c r="P148" t="inlineStr">
@@ -8162,6 +8334,7 @@
           <t>Ann &amp; Tony’s Restaurant</t>
         </is>
       </c>
+      <c r="Q148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -8200,13 +8373,13 @@
         <v>3.931</v>
       </c>
       <c r="L149" t="n">
-        <v>19.6</v>
+        <v>23</v>
       </c>
       <c r="M149" t="n">
         <v>4.046</v>
       </c>
       <c r="N149" t="n">
-        <v>26.1</v>
+        <v>28.3</v>
       </c>
       <c r="O149" t="inlineStr"/>
       <c r="P149" t="inlineStr">
@@ -8214,6 +8387,7 @@
           <t>Patricia's of Morris Park</t>
         </is>
       </c>
+      <c r="Q149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -8252,13 +8426,13 @@
         <v>3.867</v>
       </c>
       <c r="L150" t="n">
-        <v>11.1</v>
+        <v>12.5</v>
       </c>
       <c r="M150" t="n">
         <v>4.238</v>
       </c>
       <c r="N150" t="n">
-        <v>53.6</v>
+        <v>54.6</v>
       </c>
       <c r="O150" t="inlineStr"/>
       <c r="P150" t="inlineStr">
@@ -8266,6 +8440,7 @@
           <t>Emilio's of Morris Park</t>
         </is>
       </c>
+      <c r="Q150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -8304,13 +8479,13 @@
         <v>4.071</v>
       </c>
       <c r="L151" t="n">
-        <v>57.5</v>
+        <v>59.9</v>
       </c>
       <c r="M151" t="n">
         <v>4.19</v>
       </c>
       <c r="N151" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O151" t="inlineStr"/>
       <c r="P151" t="inlineStr">
@@ -8318,6 +8493,7 @@
           <t>Pine Restaurant</t>
         </is>
       </c>
+      <c r="Q151" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -8356,7 +8532,7 @@
         <v>4.343</v>
       </c>
       <c r="L152" t="n">
-        <v>93.5</v>
+        <v>94.09999999999999</v>
       </c>
       <c r="M152" t="n">
         <v>5.155</v>
@@ -8370,6 +8546,7 @@
           <t>Louie &amp; Ernie's Pizza</t>
         </is>
       </c>
+      <c r="Q152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -8422,6 +8599,7 @@
           <t>Sammy's Fish Box</t>
         </is>
       </c>
+      <c r="Q153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -8460,13 +8638,13 @@
         <v>3.934</v>
       </c>
       <c r="L154" t="n">
-        <v>21.6</v>
+        <v>25</v>
       </c>
       <c r="M154" t="n">
         <v>4.312</v>
       </c>
       <c r="N154" t="n">
-        <v>63.4</v>
+        <v>64.5</v>
       </c>
       <c r="O154" t="inlineStr"/>
       <c r="P154" t="inlineStr">
@@ -8474,6 +8652,7 @@
           <t>Beccofino</t>
         </is>
       </c>
+      <c r="Q154" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -8512,13 +8691,13 @@
         <v>3.935</v>
       </c>
       <c r="L155" t="n">
-        <v>22.2</v>
+        <v>25.7</v>
       </c>
       <c r="M155" t="n">
         <v>4.312</v>
       </c>
       <c r="N155" t="n">
-        <v>64.09999999999999</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="O155" t="inlineStr"/>
       <c r="P155" t="inlineStr">
@@ -8526,6 +8705,7 @@
           <t>Fratelli Italian Restaurant</t>
         </is>
       </c>
+      <c r="Q155" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>